<commit_message>
Add breadcrumbs, carousel, tabs blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 24
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="223">
   <si>
     <t>_reportFile</t>
   </si>
@@ -184,36 +184,39 @@
     <t>us/en/adventures/bali-surf-camp.report.json</t>
   </si>
   <si>
+    <t>["breadcrumbs","carousel","tabs"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-09-18T16:13:10.636Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.html.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>2026-09-16T16:56:38.096Z</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
     <t>["carousel","columns"]</t>
   </si>
   <si>
-    <t>us/en/adventures/bali-surf-camp</t>
-  </si>
-  <si>
-    <t>adventure-detail</t>
-  </si>
-  <si>
-    <t>2026-09-16T17:00:57.404Z</t>
-  </si>
-  <si>
-    <t>Bali Surf Camp</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.html.report.json</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.html</t>
-  </si>
-  <si>
-    <t>2026-09-16T16:56:38.096Z</t>
-  </si>
-  <si>
-    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
-  </si>
-  <si>
-    <t>us/en/adventures/beervana-portland.report.json</t>
-  </si>
-  <si>
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
@@ -583,7 +586,7 @@
     <t>article-detail</t>
   </si>
   <si>
-    <t>2026-09-16T12:16:42.246Z</t>
+    <t>2026-09-16T17:02:18.995Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -607,7 +610,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-16T12:16:55.409Z</t>
+    <t>2026-09-16T17:02:35.164Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -631,7 +634,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-16T12:16:47.491Z</t>
+    <t>2026-09-16T17:02:24.085Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -655,7 +658,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-16T12:16:51.582Z</t>
+    <t>2026-09-16T17:02:30.292Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -679,7 +682,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-16T12:16:37.135Z</t>
+    <t>2026-09-16T17:02:13.113Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -1374,7 +1377,7 @@
         <v>64</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
@@ -1383,7 +1386,7 @@
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
@@ -1392,10 +1395,10 @@
         <v>57</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J10" t="s">
         <v>63</v>
@@ -1403,7 +1406,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B11" t="s">
         <v>12</v>
@@ -1415,7 +1418,7 @@
         <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F11" t="s">
         <v>51</v>
@@ -1424,21 +1427,21 @@
         <v>12</v>
       </c>
       <c r="H11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I11" t="s">
         <v>12</v>
       </c>
       <c r="J11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
@@ -1447,7 +1450,7 @@
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F12" t="s">
         <v>14</v>
@@ -1456,18 +1459,18 @@
         <v>57</v>
       </c>
       <c r="H12" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>12</v>
@@ -1479,7 +1482,7 @@
         <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
         <v>51</v>
@@ -1488,21 +1491,21 @@
         <v>12</v>
       </c>
       <c r="H13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
       </c>
       <c r="J13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
@@ -1511,7 +1514,7 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
         <v>14</v>
@@ -1520,18 +1523,18 @@
         <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="J14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
         <v>12</v>
@@ -1543,7 +1546,7 @@
         <v>49</v>
       </c>
       <c r="E15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
         <v>51</v>
@@ -1552,21 +1555,21 @@
         <v>12</v>
       </c>
       <c r="H15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I15" t="s">
         <v>12</v>
       </c>
       <c r="J15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
         <v>12</v>
@@ -1575,7 +1578,7 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
@@ -1584,18 +1587,18 @@
         <v>57</v>
       </c>
       <c r="H16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
         <v>12</v>
@@ -1607,7 +1610,7 @@
         <v>49</v>
       </c>
       <c r="E17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F17" t="s">
         <v>51</v>
@@ -1616,21 +1619,21 @@
         <v>12</v>
       </c>
       <c r="H17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="I17" t="s">
         <v>12</v>
       </c>
       <c r="J17" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -1639,7 +1642,7 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
@@ -1648,18 +1651,18 @@
         <v>57</v>
       </c>
       <c r="H18" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I18" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="J18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
         <v>12</v>
@@ -1671,7 +1674,7 @@
         <v>49</v>
       </c>
       <c r="E19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F19" t="s">
         <v>51</v>
@@ -1680,21 +1683,21 @@
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I19" t="s">
         <v>12</v>
       </c>
       <c r="J19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -1703,7 +1706,7 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
@@ -1712,18 +1715,18 @@
         <v>57</v>
       </c>
       <c r="H20" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B21" t="s">
         <v>12</v>
@@ -1735,7 +1738,7 @@
         <v>49</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F21" t="s">
         <v>51</v>
@@ -1744,21 +1747,21 @@
         <v>12</v>
       </c>
       <c r="H21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I21" t="s">
         <v>12</v>
       </c>
       <c r="J21" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B22" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -1767,7 +1770,7 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
@@ -1776,18 +1779,18 @@
         <v>57</v>
       </c>
       <c r="H22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I22" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B23" t="s">
         <v>12</v>
@@ -1799,7 +1802,7 @@
         <v>49</v>
       </c>
       <c r="E23" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F23" t="s">
         <v>51</v>
@@ -1808,21 +1811,21 @@
         <v>12</v>
       </c>
       <c r="H23" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I23" t="s">
         <v>12</v>
       </c>
       <c r="J23" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -1831,7 +1834,7 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F24" t="s">
         <v>14</v>
@@ -1840,18 +1843,18 @@
         <v>57</v>
       </c>
       <c r="H24" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I24" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J24" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B25" t="s">
         <v>12</v>
@@ -1863,7 +1866,7 @@
         <v>49</v>
       </c>
       <c r="E25" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F25" t="s">
         <v>51</v>
@@ -1872,21 +1875,21 @@
         <v>12</v>
       </c>
       <c r="H25" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I25" t="s">
         <v>12</v>
       </c>
       <c r="J25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B26" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -1895,7 +1898,7 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
@@ -1904,18 +1907,18 @@
         <v>57</v>
       </c>
       <c r="H26" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B27" t="s">
         <v>12</v>
@@ -1927,7 +1930,7 @@
         <v>49</v>
       </c>
       <c r="E27" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F27" t="s">
         <v>51</v>
@@ -1936,21 +1939,21 @@
         <v>12</v>
       </c>
       <c r="H27" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I27" t="s">
         <v>12</v>
       </c>
       <c r="J27" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -1959,7 +1962,7 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
@@ -1968,18 +1971,18 @@
         <v>57</v>
       </c>
       <c r="H28" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I28" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="J28" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B29" t="s">
         <v>12</v>
@@ -1991,7 +1994,7 @@
         <v>49</v>
       </c>
       <c r="E29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F29" t="s">
         <v>51</v>
@@ -2000,21 +2003,21 @@
         <v>12</v>
       </c>
       <c r="H29" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I29" t="s">
         <v>12</v>
       </c>
       <c r="J29" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2023,7 +2026,7 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
@@ -2032,18 +2035,18 @@
         <v>57</v>
       </c>
       <c r="H30" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I30" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="J30" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B31" t="s">
         <v>12</v>
@@ -2055,7 +2058,7 @@
         <v>49</v>
       </c>
       <c r="E31" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F31" t="s">
         <v>51</v>
@@ -2064,21 +2067,21 @@
         <v>12</v>
       </c>
       <c r="H31" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I31" t="s">
         <v>12</v>
       </c>
       <c r="J31" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2087,7 +2090,7 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
@@ -2096,18 +2099,18 @@
         <v>57</v>
       </c>
       <c r="H32" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I32" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J32" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B33" t="s">
         <v>12</v>
@@ -2119,7 +2122,7 @@
         <v>49</v>
       </c>
       <c r="E33" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F33" t="s">
         <v>51</v>
@@ -2128,21 +2131,21 @@
         <v>12</v>
       </c>
       <c r="H33" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I33" t="s">
         <v>12</v>
       </c>
       <c r="J33" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B34" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2151,7 +2154,7 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
@@ -2160,18 +2163,18 @@
         <v>57</v>
       </c>
       <c r="H34" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I34" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="J34" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B35" t="s">
         <v>12</v>
@@ -2183,7 +2186,7 @@
         <v>49</v>
       </c>
       <c r="E35" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F35" t="s">
         <v>51</v>
@@ -2192,21 +2195,21 @@
         <v>12</v>
       </c>
       <c r="H35" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I35" t="s">
         <v>12</v>
       </c>
       <c r="J35" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B36" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2215,7 +2218,7 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
@@ -2224,18 +2227,18 @@
         <v>57</v>
       </c>
       <c r="H36" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I36" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="J36" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B37" t="s">
         <v>12</v>
@@ -2247,7 +2250,7 @@
         <v>49</v>
       </c>
       <c r="E37" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F37" t="s">
         <v>51</v>
@@ -2256,21 +2259,21 @@
         <v>12</v>
       </c>
       <c r="H37" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I37" t="s">
         <v>12</v>
       </c>
       <c r="J37" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -2279,7 +2282,7 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
@@ -2288,18 +2291,18 @@
         <v>57</v>
       </c>
       <c r="H38" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I38" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="J38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B39" t="s">
         <v>12</v>
@@ -2311,7 +2314,7 @@
         <v>49</v>
       </c>
       <c r="E39" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F39" t="s">
         <v>51</v>
@@ -2320,21 +2323,21 @@
         <v>12</v>
       </c>
       <c r="H39" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I39" t="s">
         <v>12</v>
       </c>
       <c r="J39" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B40" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -2343,27 +2346,27 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H40" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I40" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J40" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" t="s">
         <v>12</v>
@@ -2375,7 +2378,7 @@
         <v>49</v>
       </c>
       <c r="E41" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F41" t="s">
         <v>51</v>
@@ -2384,21 +2387,21 @@
         <v>12</v>
       </c>
       <c r="H41" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="I41" t="s">
         <v>12</v>
       </c>
       <c r="J41" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B42" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -2407,27 +2410,27 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H42" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I42" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J42" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B43" t="s">
         <v>12</v>
@@ -2439,7 +2442,7 @@
         <v>49</v>
       </c>
       <c r="E43" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F43" t="s">
         <v>51</v>
@@ -2448,21 +2451,21 @@
         <v>12</v>
       </c>
       <c r="H43" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="I43" t="s">
         <v>12</v>
       </c>
       <c r="J43" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B44" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -2471,27 +2474,27 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H44" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I44" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J44" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B45" t="s">
         <v>12</v>
@@ -2503,7 +2506,7 @@
         <v>49</v>
       </c>
       <c r="E45" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F45" t="s">
         <v>51</v>
@@ -2512,21 +2515,21 @@
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
       </c>
       <c r="J45" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B46" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -2535,27 +2538,27 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H46" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I46" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J46" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B47" t="s">
         <v>12</v>
@@ -2567,7 +2570,7 @@
         <v>49</v>
       </c>
       <c r="E47" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F47" t="s">
         <v>51</v>
@@ -2576,21 +2579,21 @@
         <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I47" t="s">
         <v>12</v>
       </c>
       <c r="J47" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B48" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C48" t="s">
         <v>12</v>
@@ -2599,22 +2602,22 @@
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F48" t="s">
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H48" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I48" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J48" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add adventure-list, hero blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 49
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="710" uniqueCount="319">
   <si>
     <t>_reportFile</t>
   </si>
@@ -94,7 +94,7 @@
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["teaser","adventure-list"]</t>
+    <t>["hero","adventure-list","adventure-list"]</t>
   </si>
   <si>
     <t>us/en/adventures</t>
@@ -103,7 +103,7 @@
     <t>adventures-landing</t>
   </si>
   <si>
-    <t>2026-09-16T12:29:18.213Z</t>
+    <t>2026-09-19T07:44:04.425Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -166,7 +166,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-09-18T17:13:49.974Z</t>
+    <t>2026-09-19T08:12:26.704Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -181,7 +181,7 @@
     <t>ca/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-18T17:13:55.313Z</t>
+    <t>2026-09-19T08:12:31.767Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -196,7 +196,7 @@
     <t>ca/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-18T17:13:59.987Z</t>
+    <t>2026-09-19T08:12:36.268Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -211,7 +211,7 @@
     <t>ca/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:04.575Z</t>
+    <t>2026-09-19T08:12:41.895Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -226,7 +226,7 @@
     <t>ca/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:08.288Z</t>
+    <t>2026-09-19T08:12:46.670Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -241,7 +241,7 @@
     <t>ca/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:14.305Z</t>
+    <t>2026-09-19T08:12:51.616Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -256,7 +256,7 @@
     <t>ca/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:19.715Z</t>
+    <t>2026-09-19T08:12:57.430Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -271,7 +271,7 @@
     <t>ca/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:25.358Z</t>
+    <t>2026-09-19T08:13:03.173Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -286,7 +286,7 @@
     <t>ca/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:29.824Z</t>
+    <t>2026-09-19T08:13:08.174Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -301,7 +301,7 @@
     <t>ca/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:36.070Z</t>
+    <t>2026-09-19T08:13:12.186Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -316,7 +316,7 @@
     <t>ca/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:42.054Z</t>
+    <t>2026-09-19T08:13:17.616Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -331,7 +331,7 @@
     <t>ca/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:46.494Z</t>
+    <t>2026-09-19T08:13:22.500Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -346,7 +346,7 @@
     <t>ca/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:51.889Z</t>
+    <t>2026-09-19T08:13:27.166Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -361,7 +361,7 @@
     <t>ca/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-18T17:14:57.107Z</t>
+    <t>2026-09-19T08:13:32.155Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -376,7 +376,7 @@
     <t>ca/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:02.508Z</t>
+    <t>2026-09-19T08:13:36.457Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -391,13 +391,97 @@
     <t>ca/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:07.400Z</t>
+    <t>2026-09-19T08:13:42.556Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
   </si>
   <si>
     <t>https://wknd.site/ca/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>["hero-article","breadcrumbs","author-bio","cards-related"]</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>article-detail</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:04.895Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:09.889Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>["hero-article","breadcrumbs","author-bio","author-bio","cards-related"]</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:24.548Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:30.433Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:36.516Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/western-australia.html</t>
   </si>
   <si>
     <t>us/en/adventures/bali-surf-camp.html.report.json</t>
@@ -433,7 +517,7 @@
     <t>us/en/adventures/bali-surf-camp</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:13.088Z</t>
+    <t>2026-09-19T08:13:47.916Z</t>
   </si>
   <si>
     <t>us/en/adventures/beervana-portland.html.report.json</t>
@@ -454,16 +538,28 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:17.953Z</t>
+    <t>2026-09-19T08:13:52.654Z</t>
   </si>
   <si>
     <t>us/en/adventures/climbing-new-zealand.html.report.json</t>
   </si>
   <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.evaluate: Error: Failed to import page: metaBlock.querySelector is not a function
+    at eval (eval at evaluate (:290:30), &lt;anonymous&gt;:29:15)
+    at async &lt;anonymous&gt;:316:30
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:691:31)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:954:22)</t>
+  </si>
+  <si>
     <t>us/en/adventures/climbing-new-zealand.html</t>
   </si>
   <si>
-    <t>2026-09-16T16:58:24.666Z</t>
+    <t>2026-09-19T08:11:27.693Z</t>
   </si>
   <si>
     <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
@@ -475,7 +571,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:24.088Z</t>
+    <t>2026-09-19T08:13:57.577Z</t>
   </si>
   <si>
     <t>us/en/adventures/colorado-rock-climbing.html.report.json</t>
@@ -496,7 +592,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:29.088Z</t>
+    <t>2026-09-19T08:14:03.998Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-southern-utah.html.report.json</t>
@@ -517,7 +613,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:33.231Z</t>
+    <t>2026-09-19T08:14:08.228Z</t>
   </si>
   <si>
     <t>us/en/adventures/cycling-tuscany.html.report.json</t>
@@ -538,7 +634,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:39.061Z</t>
+    <t>2026-09-19T08:14:13.619Z</t>
   </si>
   <si>
     <t>us/en/adventures/downhill-skiing-wyoming.html.report.json</t>
@@ -559,7 +655,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:44.532Z</t>
+    <t>2026-09-19T08:14:17.521Z</t>
   </si>
   <si>
     <t>us/en/adventures/gastronomic-marais-tour.html.report.json</t>
@@ -580,7 +676,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:48.415Z</t>
+    <t>2026-09-19T08:14:22.816Z</t>
   </si>
   <si>
     <t>us/en/adventures/napa-wine-tasting.html.report.json</t>
@@ -601,7 +697,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-09-18T17:15:53.895Z</t>
+    <t>2026-09-19T08:14:28.018Z</t>
   </si>
   <si>
     <t>us/en/adventures/riverside-camping-australia.html.report.json</t>
@@ -622,7 +718,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:00.077Z</t>
+    <t>2026-09-19T08:14:34.058Z</t>
   </si>
   <si>
     <t>us/en/adventures/ski-touring-mont-blanc.html.report.json</t>
@@ -643,7 +739,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:04.133Z</t>
+    <t>2026-09-19T08:14:39.516Z</t>
   </si>
   <si>
     <t>us/en/adventures/surf-camp-costa-rica.html.report.json</t>
@@ -664,7 +760,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:07.950Z</t>
+    <t>2026-09-19T08:14:45.045Z</t>
   </si>
   <si>
     <t>us/en/adventures/tahoe-skiing.html.report.json</t>
@@ -685,7 +781,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:12.574Z</t>
+    <t>2026-09-19T08:14:49.545Z</t>
   </si>
   <si>
     <t>us/en/adventures/west-coast-cycling.html.report.json</t>
@@ -706,7 +802,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:17.884Z</t>
+    <t>2026-09-19T08:14:53.826Z</t>
   </si>
   <si>
     <t>us/en/adventures/whistler-mountain-biking.html.report.json</t>
@@ -727,7 +823,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:22.722Z</t>
+    <t>2026-09-19T08:14:59.259Z</t>
   </si>
   <si>
     <t>us/en/adventures/yosemite-backpacking.html.report.json</t>
@@ -748,7 +844,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-09-18T17:16:27.596Z</t>
+    <t>2026-09-19T08:15:05.489Z</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing.html.report.json</t>
@@ -766,19 +862,10 @@
     <t>us/en/magazine/arctic-surfing.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
-    <t>article-detail</t>
-  </si>
-  <si>
-    <t>2026-09-16T17:02:18.995Z</t>
-  </si>
-  <si>
-    <t>Arctic Surfing</t>
+    <t>2026-09-18T18:26:41.149Z</t>
   </si>
   <si>
     <t>us/en/magazine/guide-la-skateparks.html.report.json</t>
@@ -799,10 +886,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:35.164Z</t>
-  </si>
-  <si>
-    <t>Ultimate Guide to LA Skateparks</t>
+    <t>2026-09-18T18:26:48.052Z</t>
   </si>
   <si>
     <t>us/en/magazine/san-diego-surf.html.report.json</t>
@@ -823,10 +907,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:24.085Z</t>
-  </si>
-  <si>
-    <t>San Diego Surf Spots</t>
+    <t>2026-09-18T18:26:54.021Z</t>
   </si>
   <si>
     <t>us/en/magazine/ski-touring.html.report.json</t>
@@ -847,10 +928,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:30.292Z</t>
-  </si>
-  <si>
-    <t>Ski Touring</t>
+    <t>2026-09-18T18:26:58.809Z</t>
   </si>
   <si>
     <t>us/en/magazine/western-australia.html.report.json</t>
@@ -871,10 +949,37 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-16T17:02:13.113Z</t>
-  </si>
-  <si>
-    <t>Western Australia</t>
+    <t>2026-09-18T18:27:04.913Z</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/alaskan-adventure</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:15.345Z</t>
+  </si>
+  <si>
+    <t>Alaskan Adventure</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/members-only/alaskan-adventure.html</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/fly-fishing-the-amazon.report.json</t>
+  </si>
+  <si>
+    <t>ca/en/magazine/members-only/fly-fishing-the-amazon</t>
+  </si>
+  <si>
+    <t>2026-09-18T18:26:19.855Z</t>
+  </si>
+  <si>
+    <t>Fly Fishing the Amazon</t>
+  </si>
+  <si>
+    <t>https://wknd.site/ca/en/magazine/members-only/fly-fishing-the-amazon.html</t>
   </si>
 </sst>
 </file>
@@ -1263,7 +1368,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1982,28 +2087,28 @@
         <v>129</v>
       </c>
       <c r="B23" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="C23" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
         <v>131</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
         <v>132</v>
       </c>
-      <c r="F23" t="s">
+      <c r="H23" t="s">
         <v>133</v>
       </c>
-      <c r="G23" t="s">
-        <v>12</v>
-      </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>134</v>
-      </c>
-      <c r="I23" t="s">
-        <v>12</v>
       </c>
       <c r="J23" t="s">
         <v>135</v>
@@ -2014,7 +2119,7 @@
         <v>136</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
@@ -2029,56 +2134,56 @@
         <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>50</v>
+        <v>132</v>
       </c>
       <c r="H24" t="s">
         <v>138</v>
       </c>
       <c r="I24" t="s">
-        <v>52</v>
+        <v>139</v>
       </c>
       <c r="J24" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>142</v>
       </c>
       <c r="C25" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F25" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G25" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="H25" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I25" t="s">
-        <v>12</v>
+        <v>145</v>
       </c>
       <c r="J25" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
-        <v>48</v>
+        <v>130</v>
       </c>
       <c r="C26" t="s">
         <v>12</v>
@@ -2087,1238 +2192,1462 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="F26" t="s">
         <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>50</v>
+        <v>132</v>
       </c>
       <c r="H26" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="I26" t="s">
-        <v>57</v>
+        <v>150</v>
       </c>
       <c r="J26" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="C27" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="F27" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="H27" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="I27" t="s">
-        <v>12</v>
+        <v>155</v>
       </c>
       <c r="J27" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C28" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E28" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="F28" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G28" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H28" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="I28" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="J28" t="s">
-        <v>149</v>
+        <v>163</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="B29" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C29" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="F29" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H29" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="I29" t="s">
-        <v>12</v>
+        <v>52</v>
       </c>
       <c r="J29" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B30" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D30" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E30" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="F30" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G30" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H30" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="I30" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
       <c r="J30" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="B31" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C31" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="F31" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H31" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="I31" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="J31" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="B32" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C32" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>176</v>
       </c>
       <c r="E32" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G32" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H32" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="I32" t="s">
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="J32" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="B33" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="F33" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H33" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="I33" t="s">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="J33" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C34" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D34" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E34" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="F34" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G34" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H34" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="I34" t="s">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="J34" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B35" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="F35" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H35" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="I35" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="J35" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="B36" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C36" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D36" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E36" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="F36" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G36" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H36" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="I36" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="J36" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="B37" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C37" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="F37" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H37" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="I37" t="s">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="J37" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C38" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D38" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E38" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="F38" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G38" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H38" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="I38" t="s">
-        <v>87</v>
+        <v>12</v>
       </c>
       <c r="J38" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C39" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D39" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="F39" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H39" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="I39" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="J39" t="s">
-        <v>191</v>
+        <v>200</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C40" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D40" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E40" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="F40" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G40" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H40" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="I40" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="J40" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="B41" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C41" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="F41" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H41" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="I41" t="s">
-        <v>12</v>
+        <v>82</v>
       </c>
       <c r="J41" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C42" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E42" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="F42" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G42" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H42" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="I42" t="s">
-        <v>97</v>
+        <v>12</v>
       </c>
       <c r="J42" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="B43" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C43" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D43" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="F43" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H43" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="I43" t="s">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="J43" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C44" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E44" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="F44" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G44" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H44" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="I44" t="s">
-        <v>102</v>
+        <v>12</v>
       </c>
       <c r="J44" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="B45" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C45" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D45" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="F45" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H45" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="I45" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="J45" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="B46" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C46" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D46" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E46" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="F46" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G46" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="I46" t="s">
-        <v>107</v>
+        <v>12</v>
       </c>
       <c r="J46" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="B47" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="F47" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H47" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="I47" t="s">
-        <v>12</v>
+        <v>97</v>
       </c>
       <c r="J47" t="s">
-        <v>219</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C48" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D48" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E48" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="F48" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G48" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H48" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="I48" t="s">
-        <v>112</v>
+        <v>12</v>
       </c>
       <c r="J48" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="B49" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C49" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="F49" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G49" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H49" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="I49" t="s">
-        <v>12</v>
+        <v>102</v>
       </c>
       <c r="J49" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="B50" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C50" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D50" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E50" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="F50" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G50" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H50" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="I50" t="s">
-        <v>117</v>
+        <v>12</v>
       </c>
       <c r="J50" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="B51" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C51" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="F51" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G51" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H51" t="s">
-        <v>232</v>
+        <v>245</v>
       </c>
       <c r="I51" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="J51" t="s">
-        <v>233</v>
+        <v>242</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="B52" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C52" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E52" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="F52" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G52" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="I52" t="s">
-        <v>122</v>
+        <v>12</v>
       </c>
       <c r="J52" t="s">
-        <v>233</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>237</v>
+        <v>250</v>
       </c>
       <c r="B53" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C53" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="F53" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G53" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H53" t="s">
-        <v>239</v>
+        <v>252</v>
       </c>
       <c r="I53" t="s">
-        <v>12</v>
+        <v>112</v>
       </c>
       <c r="J53" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="B54" t="s">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="C54" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D54" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E54" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="F54" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G54" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="H54" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="I54" t="s">
-        <v>127</v>
+        <v>12</v>
       </c>
       <c r="J54" t="s">
-        <v>240</v>
+        <v>256</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>244</v>
+        <v>257</v>
       </c>
       <c r="B55" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C55" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D55" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>245</v>
+        <v>258</v>
       </c>
       <c r="F55" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G55" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H55" t="s">
-        <v>246</v>
+        <v>259</v>
       </c>
       <c r="I55" t="s">
-        <v>12</v>
+        <v>117</v>
       </c>
       <c r="J55" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="B56" t="s">
-        <v>249</v>
+        <v>12</v>
       </c>
       <c r="C56" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D56" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E56" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="F56" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G56" t="s">
-        <v>251</v>
+        <v>12</v>
       </c>
       <c r="H56" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="I56" t="s">
-        <v>253</v>
+        <v>12</v>
       </c>
       <c r="J56" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="B57" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C57" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
       <c r="F57" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G57" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H57" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="I57" t="s">
-        <v>12</v>
+        <v>122</v>
       </c>
       <c r="J57" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="B58" t="s">
-        <v>249</v>
+        <v>12</v>
       </c>
       <c r="C58" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E58" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="F58" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G58" t="s">
-        <v>251</v>
+        <v>12</v>
       </c>
       <c r="H58" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="I58" t="s">
-        <v>261</v>
+        <v>12</v>
       </c>
       <c r="J58" t="s">
-        <v>257</v>
+        <v>270</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="B59" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="C59" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D59" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="F59" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G59" t="s">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="H59" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="I59" t="s">
-        <v>12</v>
+        <v>127</v>
       </c>
       <c r="J59" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="B60" t="s">
-        <v>249</v>
+        <v>12</v>
       </c>
       <c r="C60" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E60" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="F60" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G60" t="s">
-        <v>251</v>
+        <v>12</v>
       </c>
       <c r="H60" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="I60" t="s">
-        <v>269</v>
+        <v>12</v>
       </c>
       <c r="J60" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B61" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="C61" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D61" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="F61" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G61" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="H61" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="I61" t="s">
-        <v>12</v>
+        <v>134</v>
       </c>
       <c r="J61" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B62" t="s">
-        <v>249</v>
+        <v>12</v>
       </c>
       <c r="C62" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D62" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E62" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="F62" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G62" t="s">
-        <v>251</v>
+        <v>12</v>
       </c>
       <c r="H62" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="I62" t="s">
-        <v>277</v>
+        <v>12</v>
       </c>
       <c r="J62" t="s">
-        <v>273</v>
+        <v>284</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B63" t="s">
-        <v>12</v>
+        <v>130</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="D63" t="s">
-        <v>131</v>
+        <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="F63" t="s">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="G63" t="s">
-        <v>12</v>
+        <v>132</v>
       </c>
       <c r="H63" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="I63" t="s">
-        <v>12</v>
+        <v>139</v>
       </c>
       <c r="J63" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="B64" t="s">
-        <v>249</v>
+        <v>12</v>
       </c>
       <c r="C64" t="s">
-        <v>12</v>
+        <v>158</v>
       </c>
       <c r="D64" t="s">
-        <v>12</v>
+        <v>159</v>
       </c>
       <c r="E64" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="F64" t="s">
-        <v>14</v>
+        <v>161</v>
       </c>
       <c r="G64" t="s">
-        <v>251</v>
+        <v>12</v>
       </c>
       <c r="H64" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="I64" t="s">
-        <v>285</v>
+        <v>12</v>
       </c>
       <c r="J64" t="s">
-        <v>281</v>
+        <v>291</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>292</v>
+      </c>
+      <c r="B65" t="s">
+        <v>142</v>
+      </c>
+      <c r="C65" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" t="s">
+        <v>293</v>
+      </c>
+      <c r="F65" t="s">
+        <v>14</v>
+      </c>
+      <c r="G65" t="s">
+        <v>132</v>
+      </c>
+      <c r="H65" t="s">
+        <v>294</v>
+      </c>
+      <c r="I65" t="s">
+        <v>145</v>
+      </c>
+      <c r="J65" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>295</v>
+      </c>
+      <c r="B66" t="s">
+        <v>12</v>
+      </c>
+      <c r="C66" t="s">
+        <v>158</v>
+      </c>
+      <c r="D66" t="s">
+        <v>159</v>
+      </c>
+      <c r="E66" t="s">
+        <v>296</v>
+      </c>
+      <c r="F66" t="s">
+        <v>161</v>
+      </c>
+      <c r="G66" t="s">
+        <v>12</v>
+      </c>
+      <c r="H66" t="s">
+        <v>297</v>
+      </c>
+      <c r="I66" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>299</v>
+      </c>
+      <c r="B67" t="s">
+        <v>130</v>
+      </c>
+      <c r="C67" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>300</v>
+      </c>
+      <c r="F67" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" t="s">
+        <v>132</v>
+      </c>
+      <c r="H67" t="s">
+        <v>301</v>
+      </c>
+      <c r="I67" t="s">
+        <v>150</v>
+      </c>
+      <c r="J67" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>302</v>
+      </c>
+      <c r="B68" t="s">
+        <v>12</v>
+      </c>
+      <c r="C68" t="s">
+        <v>158</v>
+      </c>
+      <c r="D68" t="s">
+        <v>159</v>
+      </c>
+      <c r="E68" t="s">
+        <v>303</v>
+      </c>
+      <c r="F68" t="s">
+        <v>161</v>
+      </c>
+      <c r="G68" t="s">
+        <v>12</v>
+      </c>
+      <c r="H68" t="s">
+        <v>304</v>
+      </c>
+      <c r="I68" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>306</v>
+      </c>
+      <c r="B69" t="s">
+        <v>130</v>
+      </c>
+      <c r="C69" t="s">
+        <v>12</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>307</v>
+      </c>
+      <c r="F69" t="s">
+        <v>14</v>
+      </c>
+      <c r="G69" t="s">
+        <v>132</v>
+      </c>
+      <c r="H69" t="s">
+        <v>308</v>
+      </c>
+      <c r="I69" t="s">
+        <v>155</v>
+      </c>
+      <c r="J69" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>309</v>
+      </c>
+      <c r="B70" t="s">
+        <v>130</v>
+      </c>
+      <c r="C70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D70" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
+        <v>310</v>
+      </c>
+      <c r="F70" t="s">
+        <v>14</v>
+      </c>
+      <c r="G70" t="s">
+        <v>132</v>
+      </c>
+      <c r="H70" t="s">
+        <v>311</v>
+      </c>
+      <c r="I70" t="s">
+        <v>312</v>
+      </c>
+      <c r="J70" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>314</v>
+      </c>
+      <c r="B71" t="s">
+        <v>130</v>
+      </c>
+      <c r="C71" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" t="s">
+        <v>315</v>
+      </c>
+      <c r="F71" t="s">
+        <v>14</v>
+      </c>
+      <c r="G71" t="s">
+        <v>132</v>
+      </c>
+      <c r="H71" t="s">
+        <v>316</v>
+      </c>
+      <c r="I71" t="s">
+        <v>317</v>
+      </c>
+      <c r="J71" t="s">
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>